<commit_message>
edited sheet with checklists
</commit_message>
<xml_diff>
--- a/Software Testing Fundamentals/Testing sheet.xlsx
+++ b/Software Testing Fundamentals/Testing sheet.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\SkillsRepository\Software Testing Fundamentals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC28CB7-D600-4247-A4C2-7521E3118AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B03C43-ABC1-4158-8E04-66472F1DBAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Calculator.java" sheetId="1" r:id="rId1"/>
+    <sheet name="Calculator.java" sheetId="3" r:id="rId1"/>
+    <sheet name="Calculator.java devided by zero" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="15">
   <si>
     <t>+</t>
   </si>
@@ -64,6 +65,12 @@
   </si>
   <si>
     <t>✅</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>Error</t>
   </si>
 </sst>
 </file>
@@ -188,7 +195,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -482,8 +489,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{972B146B-91B6-4A36-B8A6-C3540648D2C8}">
+  <dimension ref="B2:G8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.77734375" customWidth="1"/>
@@ -595,6 +602,155 @@
         <v>12</v>
       </c>
     </row>
+    <row r="8" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="1">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:G8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
+    <col min="7" max="7" width="21.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="1">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
+        <v>6</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B5" s="1">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="1">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1">
+        <v>9</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="1">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="1">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Edited logic: program will work even after operation end
</commit_message>
<xml_diff>
--- a/Software Testing Fundamentals/Testing sheet.xlsx
+++ b/Software Testing Fundamentals/Testing sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\SkillsRepository\Software Testing Fundamentals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B03C43-ABC1-4158-8E04-66472F1DBAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABD8BDF-2E56-465E-90A3-DEED30DBD3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="16">
   <si>
     <t>+</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t>Error</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
 </sst>
 </file>
@@ -505,7 +508,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>6</v>
@@ -639,7 +642,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>6</v>

</xml_diff>